<commit_message>
clean up file locations and remove unneccessary CSVs
</commit_message>
<xml_diff>
--- a/data/processed/innovation_data.xlsx
+++ b/data/processed/innovation_data.xlsx
@@ -357,7 +357,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AK180"/>
+  <dimension ref="A1:AP180"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -544,6 +544,31 @@
       <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>2030</t>
         </is>
       </c>
     </row>
@@ -19992,7 +20017,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AK180"/>
+  <dimension ref="A1:AP180"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -20179,6 +20204,31 @@
       <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>2030</t>
         </is>
       </c>
     </row>
@@ -40510,7 +40560,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AK180"/>
+  <dimension ref="A1:AP180"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -40697,6 +40747,31 @@
       <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>2030</t>
         </is>
       </c>
     </row>
@@ -48845,7 +48920,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AK180"/>
+  <dimension ref="A1:AP180"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -49032,6 +49107,31 @@
       <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>2030</t>
         </is>
       </c>
     </row>
@@ -59988,7 +60088,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AK180"/>
+  <dimension ref="A1:AP180"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -60175,6 +60275,31 @@
       <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>2030</t>
         </is>
       </c>
     </row>
@@ -66973,7 +67098,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AK180"/>
+  <dimension ref="A1:AP180"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -67160,6 +67285,31 @@
       <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>2025</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>2030</t>
         </is>
       </c>
     </row>
@@ -77801,7 +77951,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AK180"/>
+  <dimension ref="A1:AP180"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -77990,6 +78140,31 @@
           <t>2025</t>
         </is>
       </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>2028</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>2029</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>2030</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">

</xml_diff>